<commit_message>
Add the Test Suite Files
</commit_message>
<xml_diff>
--- a/src/test/test_suite.xlsx
+++ b/src/test/test_suite.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,18 +458,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>P100040</t>
+          <t>P100098</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3929_IM-2001-0001-0001.dcm.png</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3805_IM-1915-1001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>The heart is normal in size and contour. There is no mediastinal widening. The lungs are clear bilaterally. No large pleural effusion or pneumothorax. The XXXX are intact.</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>A cardiac pacemaker/defibrillator device is redemonstration of the left chest wall with a single XXXX projecting over the right atrium and 2 leads projecting over the right ventricle. The cardiac silhouette is mildly enlarged, unchanged. No focal pulmonary consolidation. No pneumothorax. No pleural effusion. Minimal degenerative changes of the thoracic spine. .</t>
+          <t>No acute cardiopulmonary abnormalities.</t>
         </is>
       </c>
       <c r="E2" t="b">
@@ -479,18 +483,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>P100040</t>
+          <t>P100098</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3929_IM-2001-0001-0001.dcm.png</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3805_IM-1915-1001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>The heart is normal in size and contour. There is no mediastinal widening. The lungs are clear bilaterally. No large pleural effusion or pneumothorax. The XXXX are intact.</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>A cardiac pacemaker/defibrillator device is redemonstration of the left chest wall with a single XXXX projecting over the right atrium and 2 leads projecting over the right ventricle. The cardiac silhouette is mildly enlarged, unchanged. No focal pulmonary consolidation. No pneumothorax. No pleural effusion. Minimal degenerative changes of the thoracic spine. .</t>
+          <t>No acute cardiopulmonary abnormalities.</t>
         </is>
       </c>
       <c r="E3" t="b">
@@ -500,22 +508,18 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>P100088</t>
+          <t>P100083</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3972_IM-2032-2001.dcm.png</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Heart size and pulmonary vascularity appear within normal limits. Bilateral hilar fullness is present consistent with adenopathy. The appearance is unchanged. There is prominence of the interstitial markings bilaterally. These are also unchanged. No focal superimposed airspace disease is seen. No pneumothorax or pleural effusion is noted.</t>
-        </is>
-      </c>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3868_IM-1961-1001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1. Continued hilar fullness consistent with adenopathy and bilateral interstitial opacities. Stable as compared to earlier study. The changes are compatible with known diagnosis of sarcoidosis.</t>
+          <t>Heart size normal. Slight tortuous aorta. The lungs are clear. No effusions or edema</t>
         </is>
       </c>
       <c r="E4" t="b">
@@ -525,22 +529,18 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>P100088</t>
+          <t>P100083</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3972_IM-2032-2001.dcm.png</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Heart size and pulmonary vascularity appear within normal limits. Bilateral hilar fullness is present consistent with adenopathy. The appearance is unchanged. There is prominence of the interstitial markings bilaterally. These are also unchanged. No focal superimposed airspace disease is seen. No pneumothorax or pleural effusion is noted.</t>
-        </is>
-      </c>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3868_IM-1961-1001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1. Continued hilar fullness consistent with adenopathy and bilateral interstitial opacities. Stable as compared to earlier study. The changes are compatible with known diagnosis of sarcoidosis.</t>
+          <t>Heart size normal. Slight tortuous aorta. The lungs are clear. No effusions or edema</t>
         </is>
       </c>
       <c r="E5" t="b">
@@ -550,22 +550,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>P100021</t>
+          <t>P100037</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3898_IM-1978-3001.dcm.png</t>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3804_IM-1914-2001.dcm.png</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>The cardiomediastinal silhouette is normal in size and contour. No focal consolidation, pneumothorax or large pleural effusion. Normal XXXX.</t>
+          <t>Cardiomediastinal silhouette stable and within normal limits for size with unchanged atherosclerosis and tortuosity thoracic aorta. There is no focal consolidation, pneumothorax, or effusion. No acute bony abnormality. Stable left proximal humeral enchondroma versus remote bony infarct. Stable multilevel degenerative disc disease of the thoracic spine. Calcified granuloma seen anteriorly on lateral view is stable since XXXX.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Negative for acute abnormality.</t>
+          <t>No acute cardiopulmonary abnormality.</t>
         </is>
       </c>
       <c r="E6" t="b">
@@ -575,22 +575,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>P100021</t>
+          <t>P100037</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3898_IM-1978-3001.dcm.png</t>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3804_IM-1914-2001.dcm.png</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>The cardiomediastinal silhouette is normal in size and contour. No focal consolidation, pneumothorax or large pleural effusion. Normal XXXX.</t>
+          <t>Cardiomediastinal silhouette stable and within normal limits for size with unchanged atherosclerosis and tortuosity thoracic aorta. There is no focal consolidation, pneumothorax, or effusion. No acute bony abnormality. Stable left proximal humeral enchondroma versus remote bony infarct. Stable multilevel degenerative disc disease of the thoracic spine. Calcified granuloma seen anteriorly on lateral view is stable since XXXX.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Negative for acute abnormality.</t>
+          <t>No acute cardiopulmonary abnormality.</t>
         </is>
       </c>
       <c r="E7" t="b">
@@ -600,22 +600,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>P100015</t>
+          <t>P100057</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3749_IM-1874-2001.dcm.png</t>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3757_IM-1881-2001.dcm.png</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Lungs are clear bilaterally. Cardiac and mediastinal silhouettes are normal. Pulmonary vasculature is normal. No pneumothorax or pleural effusion. No acute bony abnormality.</t>
+          <t>The lungs and pleural spaces show no acute abnormality. Heart size and pulmonary vascularity within normal limits. Mild tortuosity of the descending thoracic aorta. XXXX sternotomy XXXX noted. Inferior sternotomy XXXX is disrupted.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>No acute cardiopulmonary abnormality.</t>
+          <t>1. No acute pulmonary abnormality.</t>
         </is>
       </c>
       <c r="E8" t="b">
@@ -625,22 +625,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P100015</t>
+          <t>P100057</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3749_IM-1874-2001.dcm.png</t>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3757_IM-1881-2001.dcm.png</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Lungs are clear bilaterally. Cardiac and mediastinal silhouettes are normal. Pulmonary vasculature is normal. No pneumothorax or pleural effusion. No acute bony abnormality.</t>
+          <t>The lungs and pleural spaces show no acute abnormality. Heart size and pulmonary vascularity within normal limits. Mild tortuosity of the descending thoracic aorta. XXXX sternotomy XXXX noted. Inferior sternotomy XXXX is disrupted.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>No acute cardiopulmonary abnormality.</t>
+          <t>1. No acute pulmonary abnormality.</t>
         </is>
       </c>
       <c r="E9" t="b">
@@ -650,22 +650,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>P100038</t>
+          <t>P100022</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3925_IM-1999-1004003.dcm.png</t>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3778_IM-1894-2001.dcm.png</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>The lungs are clear. There is no pleural effusion or pneumothorax. The heart is not significantly enlarged. There are calcified right hilar and mediastinal lymph XXXX. There are atherosclerotic changes of the aorta. Arthritic changes of the skeletal structures are noted.</t>
+          <t>Cardiac and mediastinal contours are within normal limits. The lungs are clear. Bony structures are intact.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>No acute pulmonary disease.</t>
+          <t>No acute findings.</t>
         </is>
       </c>
       <c r="E10" t="b">
@@ -675,25 +675,517 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>P100038</t>
+          <t>P100022</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3925_IM-1999-1004003.dcm.png</t>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3778_IM-1894-2001.dcm.png</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>The lungs are clear. There is no pleural effusion or pneumothorax. The heart is not significantly enlarged. There are calcified right hilar and mediastinal lymph XXXX. There are atherosclerotic changes of the aorta. Arthritic changes of the skeletal structures are noted.</t>
+          <t>Cardiac and mediastinal contours are within normal limits. The lungs are clear. Bony structures are intact.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>No acute pulmonary disease.</t>
+          <t>No acute findings.</t>
         </is>
       </c>
       <c r="E11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>P100087</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3969_IM-2030-2001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>The lungs hyperexpanded suggesting emphysema. The heart size and pulmonary vascularity appear within normal limits. Lungs are free of focal airspace disease. No pleural effusion or pneumothorax is seen. Osteopenia and degenerative changes are present in the spine.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>No evidence of active disease.</t>
+        </is>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>P100087</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3969_IM-2030-2001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>The lungs hyperexpanded suggesting emphysema. The heart size and pulmonary vascularity appear within normal limits. Lungs are free of focal airspace disease. No pleural effusion or pneumothorax is seen. Osteopenia and degenerative changes are present in the spine.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>No evidence of active disease.</t>
+        </is>
+      </c>
+      <c r="E13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>P100070</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3771_IM-1890-1001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Left knee. Moderately severe medial joint space narrowing and spurring. Chest. Heart size normal. Lungs clear.</t>
+        </is>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>P100070</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3771_IM-1890-1001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Left knee. Moderately severe medial joint space narrowing and spurring. Chest. Heart size normal. Lungs clear.</t>
+        </is>
+      </c>
+      <c r="E15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>P100031</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3765_IM-1884-1001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>The cardiomediastinal silhouette is within normal limits for size and contour. The lungs are normally inflated without evidence of focal airspace disease, pleural effusion, or pneumothorax. Osseous structures are within normal limits for patient age..</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1. No active disease. Specifically, no radiographic evidence for tuberculosis.</t>
+        </is>
+      </c>
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>P100031</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3765_IM-1884-1001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>The cardiomediastinal silhouette is within normal limits for size and contour. The lungs are normally inflated without evidence of focal airspace disease, pleural effusion, or pneumothorax. Osseous structures are within normal limits for patient age..</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1. No active disease. Specifically, no radiographic evidence for tuberculosis.</t>
+        </is>
+      </c>
+      <c r="E17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>P100039</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3918_IM-1992-1001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Hyperinflated lungs with mildly flattened posterior diaphragm and increased retrosternal airspace. No alveolar consolidation, no findings of pleural effusion or pulmonary edema. Heart size within normal limits. No pneumothorax.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Hyperinflated lungs, air trapping versus inspiratory XXXX.</t>
+        </is>
+      </c>
+      <c r="E18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>P100039</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3918_IM-1992-1001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Hyperinflated lungs with mildly flattened posterior diaphragm and increased retrosternal airspace. No alveolar consolidation, no findings of pleural effusion or pulmonary edema. Heart size within normal limits. No pneumothorax.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Hyperinflated lungs, air trapping versus inspiratory XXXX.</t>
+        </is>
+      </c>
+      <c r="E19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>P100091</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3982_IM-2039-1001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Normal heart size. No focal airspace consolidation, pneumothorax, pleural effusion, or pulmonary edema. No focal bony abnormality.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>No acute cardiothoracic abnormality.</t>
+        </is>
+      </c>
+      <c r="E20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>P100091</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3982_IM-2039-1001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Normal heart size. No focal airspace consolidation, pneumothorax, pleural effusion, or pulmonary edema. No focal bony abnormality.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>No acute cardiothoracic abnormality.</t>
+        </is>
+      </c>
+      <c r="E21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>P100063</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3916_IM-1991-1001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Heart size normal. Lungs XXXX clear. XXXX XXXX normal. No pneumonia, effusions, edema, pneumothorax, adenopathy, nodules or masses.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Normal chest</t>
+        </is>
+      </c>
+      <c r="E22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>P100063</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3916_IM-1991-1001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Heart size normal. Lungs XXXX clear. XXXX XXXX normal. No pneumonia, effusions, edema, pneumothorax, adenopathy, nodules or masses.</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Normal chest</t>
+        </is>
+      </c>
+      <c r="E23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>P100086</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3937_IM-2008-2001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>The heart size is upper limits of normal. The pulmonary XXXX and mediastinum are within normal limits. There is no pleural effusion or pneumothorax. There is no focal air space opacity to suggest a pneumonia. There are minimal degenerative changes of the spine.</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>No acute cardiopulmonary disease.</t>
+        </is>
+      </c>
+      <c r="E24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>P100086</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3937_IM-2008-2001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>The heart size is upper limits of normal. The pulmonary XXXX and mediastinum are within normal limits. There is no pleural effusion or pneumothorax. There is no focal air space opacity to suggest a pneumonia. There are minimal degenerative changes of the spine.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>No acute cardiopulmonary disease.</t>
+        </is>
+      </c>
+      <c r="E25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>P100018</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3971_IM-2031-2001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>The heart size and cardiomediastinal silhouette are normal. There is no focal airspace opacity, pleural effusion or pneumothorax. The bony structures are normal.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>No acute cardiopulmonary finding.</t>
+        </is>
+      </c>
+      <c r="E26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>P100018</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3971_IM-2031-2001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>The heart size and cardiomediastinal silhouette are normal. There is no focal airspace opacity, pleural effusion or pneumothorax. The bony structures are normal.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>No acute cardiopulmonary finding.</t>
+        </is>
+      </c>
+      <c r="E27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>P100097</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3957_IM-2022-2001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Cardiac and mediastinal contours are within normal limits. The lungs are clear. Bony structures are intact.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>No acute findings.</t>
+        </is>
+      </c>
+      <c r="E28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>P100097</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3957_IM-2022-2001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Cardiac and mediastinal contours are within normal limits. The lungs are clear. Bony structures are intact.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>No acute findings.</t>
+        </is>
+      </c>
+      <c r="E29" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>P100026</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3876_IM-1967-1001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>The heart is normal size. The mediastinum is unremarkable. There is no pleural effusion, pneumothorax, or focal airspace disease. There is stable mild XXXX deformity of the lower thoracic vertebral body.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>No acute cardiopulmonary abnormality.</t>
+        </is>
+      </c>
+      <c r="E30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>P100026</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>C:\Users\lokesh-g\Downloads\IU\images\images_normalized/3876_IM-1967-1001.dcm.png</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>The heart is normal size. The mediastinum is unremarkable. There is no pleural effusion, pneumothorax, or focal airspace disease. There is stable mild XXXX deformity of the lower thoracic vertebral body.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>No acute cardiopulmonary abnormality.</t>
+        </is>
+      </c>
+      <c r="E31" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>